<commit_message>
Auto update Pengadaan 2026-08-24 10:36:43
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-24).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-24).xlsx
@@ -697,7 +697,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia - 5.03.5.04.0.00.01.0000</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -739,7 +739,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politik</t>
+          <t>Badan Kesatuan Bangsa dan Politik - 8.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerah</t>
+          <t>Badan Keuangan dan Aset Daerah - 5.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -815,7 +815,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerah</t>
+          <t>Badan Penanggulangan Bencana Daerah - 1.05.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
@@ -849,7 +849,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerah</t>
+          <t>Badan Pendapatan Daerah - 5.02.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah - 5.01.5.05.0.00.01.0000</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
@@ -917,7 +917,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahraga</t>
+          <t>Dinas Kepemudaan dan Olahraga - 2.19.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -951,7 +951,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipil</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipil - 2.12.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kesehatan</t>
+          <t>Dinas Kesehatan - 1.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian - 2.16.2.20.2.21.01.0000</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidup</t>
+          <t>Dinas Lingkungan Hidup - 2.11.3.28.0.00.01.0000</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pariwisata</t>
+          <t>Dinas Pariwisata - 3.26.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruang</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruang - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatan</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatan - 1.05.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desa</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desa - 2.13.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana - 2.08.2.14.0.00.01.0000</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu - 2.18.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaan</t>
+          <t>Dinas Pendidikan dan Kebudayaan - 1.01.2.22.0.00.01.0000</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perhubungan</t>
+          <t>Dinas Perhubungan - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Pangan</t>
+          <t>Dinas Perikanan dan Ketahanan Pangan - 2.09.3.25.0.00.01.0000</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipan</t>
+          <t>Dinas Perpustakaan dan Kearsipan - 2.23.2.24.0.00.01.0000</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pertanian</t>
+          <t>Dinas Pertanian - 3.27.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan - 1.04.2.10.0.00.01.0000</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Dinas Sosial</t>
+          <t>Dinas Sosial - 1.06.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasi</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasi - 2.07.3.32.0.00.01.0000</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Inspektorat Daerah</t>
+          <t>Inspektorat Daerah - 6.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Instalasi Farmasi</t>
+          <t>Instalasi Farmasi - 1.02.0.00.0.00.01.0022</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatan</t>
+          <t>Kecamatan Arut Selatan - 7.01.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utara</t>
+          <t>Kecamatan Arut Utara - 7.01.0.00.0.00.04.0000</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lama</t>
+          <t>Kecamatan Kotawaringin Lama - 7.01.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Kumai</t>
+          <t>Kecamatan Kumai - 7.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Banteng</t>
+          <t>Kecamatan Pangkalan Banteng - 7.01.0.00.0.00.06.0000</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Lada</t>
+          <t>Kecamatan Pangkalan Lada - 7.01.0.00.0.00.05.0000</t>
         </is>
       </c>
       <c r="C42" s="8" t="n">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerah</t>
+          <t>Laboratorium Kesehatan Daerah - 1.02.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatan</t>
+          <t>Puskesmas Arut Selatan - 1.02.0.00.0.00.01.0004</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utara</t>
+          <t>Puskesmas Arut Utara - 1.02.0.00.0.00.01.0017</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jaya</t>
+          <t>Puskesmas Ipuh Bangun Jaya - 1.02.0.00.0.00.01.0021</t>
         </is>
       </c>
       <c r="C46" s="8" t="n">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulya</t>
+          <t>Puskesmas Karang Mulya - 1.02.0.00.0.00.01.0016</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lama</t>
+          <t>Puskesmas Kotawaringin Lama - 1.02.0.00.0.00.01.0019</t>
         </is>
       </c>
       <c r="C48" s="8" t="n">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Kumai</t>
+          <t>Puskesmas Kumai - 1.02.0.00.0.00.01.0010</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atas</t>
+          <t>Puskesmas Kumpai Batu Atas - 1.02.0.00.0.00.01.0008</t>
         </is>
       </c>
       <c r="C50" s="8" t="n">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejo</t>
+          <t>Puskesmas Madurejo - 1.02.0.00.0.00.01.0005</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawai</t>
+          <t>Puskesmas Mendawai - 1.02.0.00.0.00.01.0006</t>
         </is>
       </c>
       <c r="C52" s="8" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkau</t>
+          <t>Puskesmas Natai Pelingkau - 1.02.0.00.0.00.01.0007</t>
         </is>
       </c>
       <c r="C53" s="4" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjaya</t>
+          <t>Puskesmas Pandu Sanjaya - 1.02.0.00.0.00.01.0014</t>
         </is>
       </c>
       <c r="C54" s="8" t="n">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Lada</t>
+          <t>Puskesmas Pangkalan Lada - 1.02.0.00.0.00.01.0013</t>
         </is>
       </c>
       <c r="C55" s="4" t="n">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durian</t>
+          <t>Puskesmas Riam Durian - 1.02.0.00.0.00.01.0020</t>
         </is>
       </c>
       <c r="C56" s="8" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Runtu</t>
+          <t>Puskesmas Runtu - 1.02.0.00.0.00.01.0009</t>
         </is>
       </c>
       <c r="C57" s="4" t="n">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sambi</t>
+          <t>Puskesmas Sambi - 1.02.0.00.0.00.01.0018</t>
         </is>
       </c>
       <c r="C58" s="8" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggang</t>
+          <t>Puskesmas Semanggang - 1.02.0.00.0.00.01.0015</t>
         </is>
       </c>
       <c r="C59" s="4" t="n">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangit</t>
+          <t>Puskesmas Sungai Rangit - 1.02.0.00.0.00.01.0012</t>
         </is>
       </c>
       <c r="C60" s="8" t="n">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogam</t>
+          <t>Puskesmas Teluk Bogam - 1.02.0.00.0.00.01.0011</t>
         </is>
       </c>
       <c r="C61" s="4" t="n">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringin</t>
+          <t>Rumah Sakit Kutaringin - 1.02.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="C62" s="8" t="n">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddin</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddin - 1.02.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Praja</t>
+          <t>Satuan Polisi Pamong Praja - 1.05.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C64" s="8" t="n">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Sekretariat DPRD</t>
+          <t>Sekretariat DPRD - 4.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C65" s="4" t="n">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>Sekretariat Daerah</t>
+          <t>Sekretariat Daerah - 4.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C66" s="8" t="n">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia - 5.03.5.04.0.00.01.0000</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politik</t>
+          <t>Badan Kesatuan Bangsa dan Politik - 8.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerah</t>
+          <t>Badan Keuangan dan Aset Daerah - 5.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerah</t>
+          <t>Badan Penanggulangan Bencana Daerah - 1.05.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerah</t>
+          <t>Badan Pendapatan Daerah - 5.02.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah - 5.01.5.05.0.00.01.0000</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahraga</t>
+          <t>Dinas Kepemudaan dan Olahraga - 2.19.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipil</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipil - 2.12.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kesehatan</t>
+          <t>Dinas Kesehatan - 1.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian - 2.16.2.20.2.21.01.0000</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidup</t>
+          <t>Dinas Lingkungan Hidup - 2.11.3.28.0.00.01.0000</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pariwisata</t>
+          <t>Dinas Pariwisata - 3.26.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruang</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruang - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -3848,7 +3848,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatan</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatan - 1.05.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desa</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desa - 2.13.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana - 2.08.2.14.0.00.01.0000</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu - 2.18.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaan</t>
+          <t>Dinas Pendidikan dan Kebudayaan - 1.01.2.22.0.00.01.0000</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perhubungan</t>
+          <t>Dinas Perhubungan - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Pangan</t>
+          <t>Dinas Perikanan dan Ketahanan Pangan - 2.09.3.25.0.00.01.0000</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipan</t>
+          <t>Dinas Perpustakaan dan Kearsipan - 2.23.2.24.0.00.01.0000</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pertanian</t>
+          <t>Dinas Pertanian - 3.27.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan - 1.04.2.10.0.00.01.0000</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Dinas Sosial</t>
+          <t>Dinas Sosial - 1.06.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
@@ -4468,7 +4468,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasi</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasi - 2.07.3.32.0.00.01.0000</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Inspektorat Daerah</t>
+          <t>Inspektorat Daerah - 6.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
@@ -4592,7 +4592,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Instalasi Farmasi</t>
+          <t>Instalasi Farmasi - 1.02.0.00.0.00.01.0022</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
@@ -4642,7 +4642,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatan</t>
+          <t>Kecamatan Arut Selatan - 7.01.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utara</t>
+          <t>Kecamatan Arut Utara - 7.01.0.00.0.00.04.0000</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lama</t>
+          <t>Kecamatan Kotawaringin Lama - 7.01.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Kumai</t>
+          <t>Kecamatan Kumai - 7.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Banteng</t>
+          <t>Kecamatan Pangkalan Banteng - 7.01.0.00.0.00.06.0000</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Lada</t>
+          <t>Kecamatan Pangkalan Lada - 7.01.0.00.0.00.05.0000</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerah</t>
+          <t>Laboratorium Kesehatan Daerah - 1.02.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatan</t>
+          <t>Puskesmas Arut Selatan - 1.02.0.00.0.00.01.0004</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utara</t>
+          <t>Puskesmas Arut Utara - 1.02.0.00.0.00.01.0017</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jaya</t>
+          <t>Puskesmas Ipuh Bangun Jaya - 1.02.0.00.0.00.01.0021</t>
         </is>
       </c>
       <c r="C46" s="8" t="n">
@@ -5222,7 +5222,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulya</t>
+          <t>Puskesmas Karang Mulya - 1.02.0.00.0.00.01.0016</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
@@ -5284,7 +5284,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lama</t>
+          <t>Puskesmas Kotawaringin Lama - 1.02.0.00.0.00.01.0019</t>
         </is>
       </c>
       <c r="C48" s="8" t="n">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Kumai</t>
+          <t>Puskesmas Kumai - 1.02.0.00.0.00.01.0010</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atas</t>
+          <t>Puskesmas Kumpai Batu Atas - 1.02.0.00.0.00.01.0008</t>
         </is>
       </c>
       <c r="C50" s="8" t="n">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejo</t>
+          <t>Puskesmas Madurejo - 1.02.0.00.0.00.01.0005</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawai</t>
+          <t>Puskesmas Mendawai - 1.02.0.00.0.00.01.0006</t>
         </is>
       </c>
       <c r="C52" s="8" t="n">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkau</t>
+          <t>Puskesmas Natai Pelingkau - 1.02.0.00.0.00.01.0007</t>
         </is>
       </c>
       <c r="C53" s="4" t="n">
@@ -5644,7 +5644,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjaya</t>
+          <t>Puskesmas Pandu Sanjaya - 1.02.0.00.0.00.01.0014</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Lada</t>
+          <t>Puskesmas Pangkalan Lada - 1.02.0.00.0.00.01.0013</t>
         </is>
       </c>
       <c r="C55" s="4" t="n">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durian</t>
+          <t>Puskesmas Riam Durian - 1.02.0.00.0.00.01.0020</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
@@ -5846,7 +5846,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Runtu</t>
+          <t>Puskesmas Runtu - 1.02.0.00.0.00.01.0009</t>
         </is>
       </c>
       <c r="C57" s="4" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sambi</t>
+          <t>Puskesmas Sambi - 1.02.0.00.0.00.01.0018</t>
         </is>
       </c>
       <c r="C58" s="8" t="n">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggang</t>
+          <t>Puskesmas Semanggang - 1.02.0.00.0.00.01.0015</t>
         </is>
       </c>
       <c r="C59" s="4" t="n">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangit</t>
+          <t>Puskesmas Sungai Rangit - 1.02.0.00.0.00.01.0012</t>
         </is>
       </c>
       <c r="C60" s="8" t="n">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogam</t>
+          <t>Puskesmas Teluk Bogam - 1.02.0.00.0.00.01.0011</t>
         </is>
       </c>
       <c r="C61" s="4" t="n">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringin</t>
+          <t>Rumah Sakit Kutaringin - 1.02.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="C62" s="8" t="n">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddin</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddin - 1.02.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
@@ -6256,7 +6256,7 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Praja</t>
+          <t>Satuan Polisi Pamong Praja - 1.05.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C64" s="8" t="n">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Sekretariat DPRD</t>
+          <t>Sekretariat DPRD - 4.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C65" s="4" t="n">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>Sekretariat Daerah</t>
+          <t>Sekretariat Daerah - 4.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C66" s="8" t="n">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia - 5.03.5.04.0.00.01.0000</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -6801,7 +6801,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politik</t>
+          <t>Badan Kesatuan Bangsa dan Politik - 8.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -6871,7 +6871,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerah</t>
+          <t>Badan Keuangan dan Aset Daerah - 5.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerah</t>
+          <t>Badan Penanggulangan Bencana Daerah - 1.05.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerah</t>
+          <t>Badan Pendapatan Daerah - 5.02.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah - 5.01.5.05.0.00.01.0000</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
@@ -7115,7 +7115,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahraga</t>
+          <t>Dinas Kepemudaan dan Olahraga - 2.19.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -7177,7 +7177,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipil</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipil - 2.12.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kesehatan</t>
+          <t>Dinas Kesehatan - 1.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian - 2.16.2.20.2.21.01.0000</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidup</t>
+          <t>Dinas Lingkungan Hidup - 2.11.3.28.0.00.01.0000</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -7393,7 +7393,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pariwisata</t>
+          <t>Dinas Pariwisata - 3.26.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
@@ -7447,7 +7447,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruang</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruang - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatan</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatan - 1.05.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
@@ -7547,7 +7547,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desa</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desa - 2.13.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
@@ -7609,7 +7609,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana - 2.08.2.14.0.00.01.0000</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu - 2.18.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaan</t>
+          <t>Dinas Pendidikan dan Kebudayaan - 1.01.2.22.0.00.01.0000</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perhubungan</t>
+          <t>Dinas Perhubungan - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Pangan</t>
+          <t>Dinas Perikanan dan Ketahanan Pangan - 2.09.3.25.0.00.01.0000</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
@@ -7871,7 +7871,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipan</t>
+          <t>Dinas Perpustakaan dan Kearsipan - 2.23.2.24.0.00.01.0000</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pertanian</t>
+          <t>Dinas Pertanian - 3.27.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan - 1.04.2.10.0.00.01.0000</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Dinas Sosial</t>
+          <t>Dinas Sosial - 1.06.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasi</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasi - 2.07.3.32.0.00.01.0000</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
@@ -8207,7 +8207,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Inspektorat Daerah</t>
+          <t>Inspektorat Daerah - 6.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Instalasi Farmasi</t>
+          <t>Instalasi Farmasi - 1.02.0.00.0.00.01.0022</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatan</t>
+          <t>Kecamatan Arut Selatan - 7.01.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utara</t>
+          <t>Kecamatan Arut Utara - 7.01.0.00.0.00.04.0000</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lama</t>
+          <t>Kecamatan Kotawaringin Lama - 7.01.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
@@ -8497,7 +8497,7 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Kumai</t>
+          <t>Kecamatan Kumai - 7.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Banteng</t>
+          <t>Kecamatan Pangkalan Banteng - 7.01.0.00.0.00.06.0000</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Lada</t>
+          <t>Kecamatan Pangkalan Lada - 7.01.0.00.0.00.05.0000</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerah</t>
+          <t>Laboratorium Kesehatan Daerah - 1.02.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
@@ -8769,7 +8769,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatan</t>
+          <t>Puskesmas Arut Selatan - 1.02.0.00.0.00.01.0004</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
@@ -8831,7 +8831,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utara</t>
+          <t>Puskesmas Arut Utara - 1.02.0.00.0.00.01.0017</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
@@ -8893,7 +8893,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jaya</t>
+          <t>Puskesmas Ipuh Bangun Jaya - 1.02.0.00.0.00.01.0021</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -8963,7 +8963,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulya</t>
+          <t>Puskesmas Karang Mulya - 1.02.0.00.0.00.01.0016</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
@@ -9033,7 +9033,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lama</t>
+          <t>Puskesmas Kotawaringin Lama - 1.02.0.00.0.00.01.0019</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
@@ -9103,7 +9103,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Kumai</t>
+          <t>Puskesmas Kumai - 1.02.0.00.0.00.01.0010</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atas</t>
+          <t>Puskesmas Kumpai Batu Atas - 1.02.0.00.0.00.01.0008</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
@@ -9235,7 +9235,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejo</t>
+          <t>Puskesmas Madurejo - 1.02.0.00.0.00.01.0005</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawai</t>
+          <t>Puskesmas Mendawai - 1.02.0.00.0.00.01.0006</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkau</t>
+          <t>Puskesmas Natai Pelingkau - 1.02.0.00.0.00.01.0007</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjaya</t>
+          <t>Puskesmas Pandu Sanjaya - 1.02.0.00.0.00.01.0014</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
@@ -9515,7 +9515,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Lada</t>
+          <t>Puskesmas Pangkalan Lada - 1.02.0.00.0.00.01.0013</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durian</t>
+          <t>Puskesmas Riam Durian - 1.02.0.00.0.00.01.0020</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
@@ -9655,7 +9655,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Runtu</t>
+          <t>Puskesmas Runtu - 1.02.0.00.0.00.01.0009</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
@@ -9725,7 +9725,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sambi</t>
+          <t>Puskesmas Sambi - 1.02.0.00.0.00.01.0018</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
@@ -9795,7 +9795,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggang</t>
+          <t>Puskesmas Semanggang - 1.02.0.00.0.00.01.0015</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -9865,7 +9865,7 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangit</t>
+          <t>Puskesmas Sungai Rangit - 1.02.0.00.0.00.01.0012</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogam</t>
+          <t>Puskesmas Teluk Bogam - 1.02.0.00.0.00.01.0011</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringin</t>
+          <t>Rumah Sakit Kutaringin - 1.02.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
@@ -10075,7 +10075,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddin</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddin - 1.02.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
@@ -10121,7 +10121,7 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Praja</t>
+          <t>Satuan Polisi Pamong Praja - 1.05.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C64" s="8" t="n">
@@ -10183,7 +10183,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Sekretariat DPRD</t>
+          <t>Sekretariat DPRD - 4.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C65" s="4" t="n">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>Sekretariat Daerah</t>
+          <t>Sekretariat Daerah - 4.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C66" s="8" t="n">
@@ -10616,7 +10616,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia</t>
+          <t>Badan Kepegawaian dan Pengembangan Sumber Daya Manusia - 5.03.5.04.0.00.01.0000</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -10686,7 +10686,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Badan Kesatuan Bangsa dan Politik</t>
+          <t>Badan Kesatuan Bangsa dan Politik - 8.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -10756,7 +10756,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Badan Keuangan dan Aset Daerah</t>
+          <t>Badan Keuangan dan Aset Daerah - 5.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Badan Penanggulangan Bencana Daerah</t>
+          <t>Badan Penanggulangan Bencana Daerah - 1.05.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Badan Pendapatan Daerah</t>
+          <t>Badan Pendapatan Daerah - 5.02.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -10966,7 +10966,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah</t>
+          <t>Badan Perencanaan Pembangunan, Riset dan Inovasi Daerah - 5.01.5.05.0.00.01.0000</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -11036,7 +11036,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kepemudaan dan Olahraga</t>
+          <t>Dinas Kepemudaan dan Olahraga - 2.19.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Dinas Kependudukan dan Pencatatan Sipil</t>
+          <t>Dinas Kependudukan dan Pencatatan Sipil - 2.12.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -11176,7 +11176,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Dinas Kesehatan</t>
+          <t>Dinas Kesehatan - 1.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian</t>
+          <t>Dinas Komunikasi, Informatika, Statistik dan Persandian - 2.16.2.20.2.21.01.0000</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
@@ -11300,7 +11300,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Dinas Lingkungan Hidup</t>
+          <t>Dinas Lingkungan Hidup - 2.11.3.28.0.00.01.0000</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -11354,7 +11354,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pariwisata</t>
+          <t>Dinas Pariwisata - 3.26.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pekerjaan Umum dan Penataan Ruang</t>
+          <t>Dinas Pekerjaan Umum dan Penataan Ruang - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemadam Kebakaran dan Penyelamatan</t>
+          <t>Dinas Pemadam Kebakaran dan Penyelamatan - 1.05.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -11548,7 +11548,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Masyarakat dan Desa</t>
+          <t>Dinas Pemberdayaan Masyarakat dan Desa - 2.13.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana</t>
+          <t>Dinas Pemberdayaan Perempuan dan Perlindungan Anak, Pengendalian Penduduk dan Keluarga Berencana - 2.08.2.14.0.00.01.0000</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -11688,7 +11688,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu</t>
+          <t>Dinas Penanaman Modal dan Pelayanan Terpadu Satu Pintu - 2.18.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Dinas Pendidikan dan Kebudayaan</t>
+          <t>Dinas Pendidikan dan Kebudayaan - 1.01.2.22.0.00.01.0000</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
@@ -11820,7 +11820,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perhubungan</t>
+          <t>Dinas Perhubungan - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perikanan dan Ketahanan Pangan</t>
+          <t>Dinas Perikanan dan Ketahanan Pangan - 2.09.3.25.0.00.01.0000</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -11940,7 +11940,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah</t>
+          <t>Dinas Perindustrian, Perdagangan, Koperasi, Usaha Kecil dan Menengah - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
@@ -11994,7 +11994,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perpustakaan dan Kearsipan</t>
+          <t>Dinas Perpustakaan dan Kearsipan - 2.23.2.24.0.00.01.0000</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Dinas Pertanian</t>
+          <t>Dinas Pertanian - 3.27.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -12126,7 +12126,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan</t>
+          <t>Dinas Perumahan Rakyat, Kawasan Pemukiman dan Pertanahan - 1.04.2.10.0.00.01.0000</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -12196,7 +12196,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Dinas Sosial</t>
+          <t>Dinas Sosial - 1.06.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -12266,7 +12266,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Dinas Tenaga Kerja dan Transmigrasi</t>
+          <t>Dinas Tenaga Kerja dan Transmigrasi - 2.07.3.32.0.00.01.0000</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Inspektorat Daerah</t>
+          <t>Inspektorat Daerah - 6.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Instalasi Farmasi</t>
+          <t>Instalasi Farmasi - 1.02.0.00.0.00.01.0022</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Selatan</t>
+          <t>Kecamatan Arut Selatan - 7.01.0.00.0.00.02.0000</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -12546,7 +12546,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Arut Utara</t>
+          <t>Kecamatan Arut Utara - 7.01.0.00.0.00.04.0000</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
@@ -12616,7 +12616,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Kotawaringin Lama</t>
+          <t>Kecamatan Kotawaringin Lama - 7.01.0.00.0.00.03.0000</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -12686,7 +12686,7 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Kumai</t>
+          <t>Kecamatan Kumai - 7.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -12756,7 +12756,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Banteng</t>
+          <t>Kecamatan Pangkalan Banteng - 7.01.0.00.0.00.06.0000</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -12826,7 +12826,7 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Kecamatan Pangkalan Lada</t>
+          <t>Kecamatan Pangkalan Lada - 7.01.0.00.0.00.05.0000</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
@@ -12896,7 +12896,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Laboratorium Kesehatan Daerah</t>
+          <t>Laboratorium Kesehatan Daerah - 1.02.0.00.0.00.01.0003</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -12966,7 +12966,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Selatan</t>
+          <t>Puskesmas Arut Selatan - 1.02.0.00.0.00.01.0004</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
@@ -13036,7 +13036,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Arut Utara</t>
+          <t>Puskesmas Arut Utara - 1.02.0.00.0.00.01.0017</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
@@ -13106,7 +13106,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Ipuh Bangun Jaya</t>
+          <t>Puskesmas Ipuh Bangun Jaya - 1.02.0.00.0.00.01.0021</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -13176,7 +13176,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Karang Mulya</t>
+          <t>Puskesmas Karang Mulya - 1.02.0.00.0.00.01.0016</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kotawaringin Lama</t>
+          <t>Puskesmas Kotawaringin Lama - 1.02.0.00.0.00.01.0019</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
@@ -13316,7 +13316,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Kumai</t>
+          <t>Puskesmas Kumai - 1.02.0.00.0.00.01.0010</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Kumpai Batu Atas</t>
+          <t>Puskesmas Kumpai Batu Atas - 1.02.0.00.0.00.01.0008</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Madurejo</t>
+          <t>Puskesmas Madurejo - 1.02.0.00.0.00.01.0005</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
@@ -13526,7 +13526,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Mendawai</t>
+          <t>Puskesmas Mendawai - 1.02.0.00.0.00.01.0006</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Natai Pelingkau</t>
+          <t>Puskesmas Natai Pelingkau - 1.02.0.00.0.00.01.0007</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Pandu Sanjaya</t>
+          <t>Puskesmas Pandu Sanjaya - 1.02.0.00.0.00.01.0014</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
@@ -13736,7 +13736,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Pangkalan Lada</t>
+          <t>Puskesmas Pangkalan Lada - 1.02.0.00.0.00.01.0013</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -13806,7 +13806,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Riam Durian</t>
+          <t>Puskesmas Riam Durian - 1.02.0.00.0.00.01.0020</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
@@ -13876,7 +13876,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Runtu</t>
+          <t>Puskesmas Runtu - 1.02.0.00.0.00.01.0009</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
@@ -13946,7 +13946,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sambi</t>
+          <t>Puskesmas Sambi - 1.02.0.00.0.00.01.0018</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
@@ -14016,7 +14016,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Semanggang</t>
+          <t>Puskesmas Semanggang - 1.02.0.00.0.00.01.0015</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Puskesmas Sungai Rangit</t>
+          <t>Puskesmas Sungai Rangit - 1.02.0.00.0.00.01.0012</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
@@ -14156,7 +14156,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Puskesmas Teluk Bogam</t>
+          <t>Puskesmas Teluk Bogam - 1.02.0.00.0.00.01.0011</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
@@ -14226,7 +14226,7 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>Rumah Sakit Kutaringin</t>
+          <t>Rumah Sakit Kutaringin - 1.02.0.00.0.00.01.0002</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
@@ -14296,7 +14296,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Rumah Sakit Umum Daerah Sultan Imanuddin</t>
+          <t>Rumah Sakit Umum Daerah Sultan Imanuddin - 1.02.0.00.0.00.01.0001</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
@@ -14346,7 +14346,7 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>Satuan Polisi Pamong Praja</t>
+          <t>Satuan Polisi Pamong Praja - 1.05.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Sekretariat DPRD</t>
+          <t>Sekretariat DPRD - 4.02.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -14486,7 +14486,7 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>Sekretariat Daerah</t>
+          <t>Sekretariat Daerah - 4.01.0.00.0.00.01.0000</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">

</xml_diff>